<commit_message>
Correction : panneaux dessinés en lignes (LINE) ajoutés
12 panneaux manquants identifiés car dessinés avec 4 lignes
individuelles au lieu de LWPOLYLINE dans le DXF :
- 542×2550mm RDC (Façade Est) × 1
- 542×3650mm N1 (Façade Est) × 1
- 4268×1064mm Bandeau Haut (Façade Ouest) × 5
- 4268×1064mm Bandeau Haut (Façade Est) × 5

Surface totale corrigée : 479 m² → 527.955 m²
Total panneaux : 234 → 246

https://claude.ai/code/session_01XEBC19dXnMVpZDyxAKSfaP
</commit_message>
<xml_diff>
--- a/Panneaux_Trespa_Detail.xlsx
+++ b/Panneaux_Trespa_Detail.xlsx
@@ -561,22 +561,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G65"/>
+  <dimension ref="A1:G68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>RÉCAPITULATIF - Panneaux Trespa Beauchamp</t>
+          <t>RÉCAPITULATIF — Panneaux Trespa Beauchamp</t>
         </is>
       </c>
     </row>
@@ -588,32 +588,32 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Largeur façade (mm)</t>
+          <t>Larg. (mm)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Hauteur panneau (mm)</t>
+          <t>Haut. (mm)</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>F. Nord</t>
+          <t>F.Nord</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>F. Ouest</t>
+          <t>F.Ouest</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>F. Est</t>
+          <t>F.Est</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>F. Sud</t>
+          <t>F.Sud</t>
         </is>
       </c>
     </row>
@@ -693,27 +693,27 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>Dessus fenêtre N1</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="n">
-        <v>788</v>
-      </c>
-      <c r="C6" s="6" t="n">
-        <v>1007.9</v>
-      </c>
-      <c r="D6" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="G6" s="6" t="n">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Bandeau Haut</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>4268</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>1064</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="G6" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -727,16 +727,16 @@
         <v>788</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>1008</v>
+        <v>1007.9</v>
       </c>
       <c r="D7" s="6" t="n">
         <v>0</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G7" s="6" t="n">
         <v>0</v>
@@ -749,19 +749,19 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>984</v>
+        <v>788</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>1007.9</v>
+        <v>1008</v>
       </c>
       <c r="D8" s="6" t="n">
         <v>0</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G8" s="6" t="n">
         <v>0</v>
@@ -777,16 +777,16 @@
         <v>984</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>1008</v>
+        <v>1007.9</v>
       </c>
       <c r="D9" s="6" t="n">
         <v>0</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G9" s="6" t="n">
         <v>0</v>
@@ -799,22 +799,22 @@
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>1134</v>
+        <v>984</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>1007.9</v>
+        <v>1008</v>
       </c>
       <c r="D10" s="6" t="n">
         <v>0</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F10" s="6" t="n">
         <v>0</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -824,47 +824,47 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
+        <v>1134</v>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>1007.9</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Dessus fenêtre N1</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n">
         <v>1584</v>
       </c>
-      <c r="C11" s="6" t="n">
+      <c r="C12" s="6" t="n">
         <v>1008</v>
       </c>
-      <c r="D11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="6" t="n">
+      <c r="D12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>Plein N1</t>
-        </is>
-      </c>
-      <c r="B12" s="8" t="n">
-        <v>296</v>
-      </c>
-      <c r="C12" s="8" t="n">
-        <v>3650</v>
-      </c>
-      <c r="D12" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" s="8" t="n">
-        <v>2</v>
+      <c r="F12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -874,22 +874,22 @@
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>445</v>
+        <v>296</v>
       </c>
       <c r="C13" s="8" t="n">
-        <v>3651.2</v>
+        <v>3650</v>
       </c>
       <c r="D13" s="8" t="n">
         <v>0</v>
       </c>
       <c r="E13" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F13" s="8" t="n">
         <v>0</v>
       </c>
       <c r="G13" s="8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
@@ -899,10 +899,10 @@
         </is>
       </c>
       <c r="B14" s="8" t="n">
-        <v>491</v>
+        <v>445</v>
       </c>
       <c r="C14" s="8" t="n">
-        <v>3650</v>
+        <v>3651.2</v>
       </c>
       <c r="D14" s="8" t="n">
         <v>0</v>
@@ -924,7 +924,7 @@
         </is>
       </c>
       <c r="B15" s="8" t="n">
-        <v>620</v>
+        <v>491</v>
       </c>
       <c r="C15" s="8" t="n">
         <v>3650</v>
@@ -949,7 +949,7 @@
         </is>
       </c>
       <c r="B16" s="8" t="n">
-        <v>650.5</v>
+        <v>542</v>
       </c>
       <c r="C16" s="8" t="n">
         <v>3650</v>
@@ -958,10 +958,10 @@
         <v>0</v>
       </c>
       <c r="E16" s="8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G16" s="8" t="n">
         <v>0</v>
@@ -974,7 +974,7 @@
         </is>
       </c>
       <c r="B17" s="8" t="n">
-        <v>776</v>
+        <v>620</v>
       </c>
       <c r="C17" s="8" t="n">
         <v>3650</v>
@@ -983,10 +983,10 @@
         <v>0</v>
       </c>
       <c r="E17" s="8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G17" s="8" t="n">
         <v>0</v>
@@ -999,7 +999,7 @@
         </is>
       </c>
       <c r="B18" s="8" t="n">
-        <v>777</v>
+        <v>650.5</v>
       </c>
       <c r="C18" s="8" t="n">
         <v>3650</v>
@@ -1008,10 +1008,10 @@
         <v>0</v>
       </c>
       <c r="E18" s="8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G18" s="8" t="n">
         <v>0</v>
@@ -1024,7 +1024,7 @@
         </is>
       </c>
       <c r="B19" s="8" t="n">
-        <v>778</v>
+        <v>776</v>
       </c>
       <c r="C19" s="8" t="n">
         <v>3650</v>
@@ -1033,10 +1033,10 @@
         <v>0</v>
       </c>
       <c r="E19" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="8" t="n">
         <v>1</v>
-      </c>
-      <c r="F19" s="8" t="n">
-        <v>2</v>
       </c>
       <c r="G19" s="8" t="n">
         <v>0</v>
@@ -1049,7 +1049,7 @@
         </is>
       </c>
       <c r="B20" s="8" t="n">
-        <v>821</v>
+        <v>777</v>
       </c>
       <c r="C20" s="8" t="n">
         <v>3650</v>
@@ -1058,10 +1058,10 @@
         <v>0</v>
       </c>
       <c r="E20" s="8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G20" s="8" t="n">
         <v>0</v>
@@ -1074,7 +1074,7 @@
         </is>
       </c>
       <c r="B21" s="8" t="n">
-        <v>822.3</v>
+        <v>778</v>
       </c>
       <c r="C21" s="8" t="n">
         <v>3650</v>
@@ -1083,10 +1083,10 @@
         <v>0</v>
       </c>
       <c r="E21" s="8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F21" s="8" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="G21" s="8" t="n">
         <v>0</v>
@@ -1099,7 +1099,7 @@
         </is>
       </c>
       <c r="B22" s="8" t="n">
-        <v>833</v>
+        <v>821</v>
       </c>
       <c r="C22" s="8" t="n">
         <v>3650</v>
@@ -1108,10 +1108,10 @@
         <v>0</v>
       </c>
       <c r="E22" s="8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G22" s="8" t="n">
         <v>0</v>
@@ -1124,22 +1124,22 @@
         </is>
       </c>
       <c r="B23" s="8" t="n">
-        <v>867</v>
+        <v>822.3</v>
       </c>
       <c r="C23" s="8" t="n">
         <v>3650</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="E23" s="8" t="n">
         <v>0</v>
       </c>
       <c r="F23" s="8" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G23" s="8" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -1149,7 +1149,7 @@
         </is>
       </c>
       <c r="B24" s="8" t="n">
-        <v>876</v>
+        <v>833</v>
       </c>
       <c r="C24" s="8" t="n">
         <v>3650</v>
@@ -1158,10 +1158,10 @@
         <v>0</v>
       </c>
       <c r="E24" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G24" s="8" t="n">
         <v>0</v>
@@ -1174,22 +1174,22 @@
         </is>
       </c>
       <c r="B25" s="8" t="n">
-        <v>877</v>
+        <v>867</v>
       </c>
       <c r="C25" s="8" t="n">
         <v>3650</v>
       </c>
       <c r="D25" s="8" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="E25" s="8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F25" s="8" t="n">
         <v>0</v>
       </c>
       <c r="G25" s="8" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
     </row>
     <row r="26">
@@ -1199,7 +1199,7 @@
         </is>
       </c>
       <c r="B26" s="8" t="n">
-        <v>933.5</v>
+        <v>876</v>
       </c>
       <c r="C26" s="8" t="n">
         <v>3650</v>
@@ -1208,7 +1208,7 @@
         <v>0</v>
       </c>
       <c r="E26" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F26" s="8" t="n">
         <v>0</v>
@@ -1224,7 +1224,7 @@
         </is>
       </c>
       <c r="B27" s="8" t="n">
-        <v>981</v>
+        <v>877</v>
       </c>
       <c r="C27" s="8" t="n">
         <v>3650</v>
@@ -1233,10 +1233,10 @@
         <v>0</v>
       </c>
       <c r="E27" s="8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F27" s="8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G27" s="8" t="n">
         <v>0</v>
@@ -1249,7 +1249,7 @@
         </is>
       </c>
       <c r="B28" s="8" t="n">
-        <v>983</v>
+        <v>933.5</v>
       </c>
       <c r="C28" s="8" t="n">
         <v>3650</v>
@@ -1274,7 +1274,7 @@
         </is>
       </c>
       <c r="B29" s="8" t="n">
-        <v>1028.5</v>
+        <v>981</v>
       </c>
       <c r="C29" s="8" t="n">
         <v>3650</v>
@@ -1299,7 +1299,7 @@
         </is>
       </c>
       <c r="B30" s="8" t="n">
-        <v>1037</v>
+        <v>983</v>
       </c>
       <c r="C30" s="8" t="n">
         <v>3650</v>
@@ -1324,7 +1324,7 @@
         </is>
       </c>
       <c r="B31" s="8" t="n">
-        <v>1078</v>
+        <v>1028.5</v>
       </c>
       <c r="C31" s="8" t="n">
         <v>3650</v>
@@ -1333,10 +1333,10 @@
         <v>0</v>
       </c>
       <c r="E31" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F31" s="8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G31" s="8" t="n">
         <v>0</v>
@@ -1349,71 +1349,71 @@
         </is>
       </c>
       <c r="B32" s="8" t="n">
+        <v>1037</v>
+      </c>
+      <c r="C32" s="8" t="n">
+        <v>3650</v>
+      </c>
+      <c r="D32" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F32" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>Plein N1</t>
+        </is>
+      </c>
+      <c r="B33" s="8" t="n">
+        <v>1078</v>
+      </c>
+      <c r="C33" s="8" t="n">
+        <v>3650</v>
+      </c>
+      <c r="D33" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>Plein N1</t>
+        </is>
+      </c>
+      <c r="B34" s="8" t="n">
         <v>1083</v>
       </c>
-      <c r="C32" s="8" t="n">
-        <v>3650</v>
-      </c>
-      <c r="D32" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E32" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="F32" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="G32" s="8" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="9" t="inlineStr">
-        <is>
-          <t>Dessous fenêtre N1</t>
-        </is>
-      </c>
-      <c r="B33" s="10" t="n">
-        <v>788</v>
-      </c>
-      <c r="C33" s="10" t="n">
-        <v>822</v>
-      </c>
-      <c r="D33" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E33" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="F33" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G33" s="10" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="9" t="inlineStr">
-        <is>
-          <t>Dessous fenêtre N1</t>
-        </is>
-      </c>
-      <c r="B34" s="10" t="n">
-        <v>788</v>
-      </c>
-      <c r="C34" s="10" t="n">
-        <v>822.1</v>
-      </c>
-      <c r="D34" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E34" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F34" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="G34" s="10" t="n">
+      <c r="C34" s="8" t="n">
+        <v>3650</v>
+      </c>
+      <c r="D34" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F34" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1424,19 +1424,19 @@
         </is>
       </c>
       <c r="B35" s="10" t="n">
-        <v>833</v>
+        <v>788</v>
       </c>
       <c r="C35" s="10" t="n">
-        <v>842.1</v>
+        <v>822</v>
       </c>
       <c r="D35" s="10" t="n">
         <v>0</v>
       </c>
       <c r="E35" s="10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F35" s="10" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G35" s="10" t="n">
         <v>0</v>
@@ -1449,19 +1449,19 @@
         </is>
       </c>
       <c r="B36" s="10" t="n">
-        <v>984</v>
+        <v>788</v>
       </c>
       <c r="C36" s="10" t="n">
-        <v>822</v>
+        <v>822.1</v>
       </c>
       <c r="D36" s="10" t="n">
         <v>0</v>
       </c>
       <c r="E36" s="10" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="F36" s="10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G36" s="10" t="n">
         <v>0</v>
@@ -1474,97 +1474,97 @@
         </is>
       </c>
       <c r="B37" s="10" t="n">
+        <v>833</v>
+      </c>
+      <c r="C37" s="10" t="n">
+        <v>842.1</v>
+      </c>
+      <c r="D37" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="G37" s="10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="9" t="inlineStr">
+        <is>
+          <t>Dessous fenêtre N1</t>
+        </is>
+      </c>
+      <c r="B38" s="10" t="n">
         <v>984</v>
       </c>
-      <c r="C37" s="10" t="n">
+      <c r="C38" s="10" t="n">
+        <v>822</v>
+      </c>
+      <c r="D38" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="F38" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" s="10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="9" t="inlineStr">
+        <is>
+          <t>Dessous fenêtre N1</t>
+        </is>
+      </c>
+      <c r="B39" s="10" t="n">
+        <v>984</v>
+      </c>
+      <c r="C39" s="10" t="n">
         <v>822.1</v>
       </c>
-      <c r="D37" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E37" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F37" s="10" t="n">
+      <c r="D39" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="G37" s="10" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="11" t="inlineStr">
+      <c r="G39" s="10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="11" t="inlineStr">
         <is>
           <t>Dessus porte N1</t>
         </is>
       </c>
-      <c r="B38" s="12" t="n">
+      <c r="B40" s="12" t="n">
         <v>1134</v>
       </c>
-      <c r="C38" s="12" t="n">
+      <c r="C40" s="12" t="n">
         <v>492.1</v>
       </c>
-      <c r="D38" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E38" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F38" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G38" s="12" t="n">
+      <c r="D40" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" s="12" t="n">
         <v>1</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="13" t="inlineStr">
-        <is>
-          <t>Plein RDC</t>
-        </is>
-      </c>
-      <c r="B39" s="14" t="n">
-        <v>296</v>
-      </c>
-      <c r="C39" s="14" t="n">
-        <v>2550</v>
-      </c>
-      <c r="D39" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E39" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F39" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G39" s="14" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="13" t="inlineStr">
-        <is>
-          <t>Plein RDC</t>
-        </is>
-      </c>
-      <c r="B40" s="14" t="n">
-        <v>445</v>
-      </c>
-      <c r="C40" s="14" t="n">
-        <v>2550</v>
-      </c>
-      <c r="D40" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E40" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="F40" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G40" s="14" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -1574,7 +1574,7 @@
         </is>
       </c>
       <c r="B41" s="14" t="n">
-        <v>491</v>
+        <v>296</v>
       </c>
       <c r="C41" s="14" t="n">
         <v>2550</v>
@@ -1583,13 +1583,13 @@
         <v>0</v>
       </c>
       <c r="E41" s="14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F41" s="14" t="n">
         <v>0</v>
       </c>
       <c r="G41" s="14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="42">
@@ -1599,7 +1599,7 @@
         </is>
       </c>
       <c r="B42" s="14" t="n">
-        <v>620</v>
+        <v>445</v>
       </c>
       <c r="C42" s="14" t="n">
         <v>2550</v>
@@ -1624,7 +1624,7 @@
         </is>
       </c>
       <c r="B43" s="14" t="n">
-        <v>650.5</v>
+        <v>491</v>
       </c>
       <c r="C43" s="14" t="n">
         <v>2550</v>
@@ -1633,7 +1633,7 @@
         <v>0</v>
       </c>
       <c r="E43" s="14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F43" s="14" t="n">
         <v>0</v>
@@ -1649,7 +1649,7 @@
         </is>
       </c>
       <c r="B44" s="14" t="n">
-        <v>776</v>
+        <v>542</v>
       </c>
       <c r="C44" s="14" t="n">
         <v>2550</v>
@@ -1674,7 +1674,7 @@
         </is>
       </c>
       <c r="B45" s="14" t="n">
-        <v>777</v>
+        <v>620</v>
       </c>
       <c r="C45" s="14" t="n">
         <v>2550</v>
@@ -1683,10 +1683,10 @@
         <v>0</v>
       </c>
       <c r="E45" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F45" s="14" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G45" s="14" t="n">
         <v>0</v>
@@ -1699,7 +1699,7 @@
         </is>
       </c>
       <c r="B46" s="14" t="n">
-        <v>778</v>
+        <v>650.5</v>
       </c>
       <c r="C46" s="14" t="n">
         <v>2550</v>
@@ -1708,10 +1708,10 @@
         <v>0</v>
       </c>
       <c r="E46" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F46" s="14" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G46" s="14" t="n">
         <v>0</v>
@@ -1724,7 +1724,7 @@
         </is>
       </c>
       <c r="B47" s="14" t="n">
-        <v>821</v>
+        <v>776</v>
       </c>
       <c r="C47" s="14" t="n">
         <v>2550</v>
@@ -1733,10 +1733,10 @@
         <v>0</v>
       </c>
       <c r="E47" s="14" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F47" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G47" s="14" t="n">
         <v>0</v>
@@ -1749,7 +1749,7 @@
         </is>
       </c>
       <c r="B48" s="14" t="n">
-        <v>822.3</v>
+        <v>777</v>
       </c>
       <c r="C48" s="14" t="n">
         <v>2550</v>
@@ -1761,7 +1761,7 @@
         <v>0</v>
       </c>
       <c r="F48" s="14" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="G48" s="14" t="n">
         <v>0</v>
@@ -1774,7 +1774,7 @@
         </is>
       </c>
       <c r="B49" s="14" t="n">
-        <v>833</v>
+        <v>778</v>
       </c>
       <c r="C49" s="14" t="n">
         <v>2550</v>
@@ -1783,10 +1783,10 @@
         <v>0</v>
       </c>
       <c r="E49" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F49" s="14" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G49" s="14" t="n">
         <v>0</v>
@@ -1799,22 +1799,22 @@
         </is>
       </c>
       <c r="B50" s="14" t="n">
-        <v>867</v>
+        <v>821</v>
       </c>
       <c r="C50" s="14" t="n">
         <v>2550</v>
       </c>
       <c r="D50" s="14" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="E50" s="14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F50" s="14" t="n">
         <v>0</v>
       </c>
       <c r="G50" s="14" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51">
@@ -1824,7 +1824,7 @@
         </is>
       </c>
       <c r="B51" s="14" t="n">
-        <v>876</v>
+        <v>822.3</v>
       </c>
       <c r="C51" s="14" t="n">
         <v>2550</v>
@@ -1833,10 +1833,10 @@
         <v>0</v>
       </c>
       <c r="E51" s="14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F51" s="14" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G51" s="14" t="n">
         <v>0</v>
@@ -1849,7 +1849,7 @@
         </is>
       </c>
       <c r="B52" s="14" t="n">
-        <v>877</v>
+        <v>833</v>
       </c>
       <c r="C52" s="14" t="n">
         <v>2550</v>
@@ -1858,10 +1858,10 @@
         <v>0</v>
       </c>
       <c r="E52" s="14" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F52" s="14" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G52" s="14" t="n">
         <v>0</v>
@@ -1874,22 +1874,22 @@
         </is>
       </c>
       <c r="B53" s="14" t="n">
-        <v>933.5</v>
+        <v>867</v>
       </c>
       <c r="C53" s="14" t="n">
         <v>2550</v>
       </c>
       <c r="D53" s="14" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="E53" s="14" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F53" s="14" t="n">
         <v>0</v>
       </c>
       <c r="G53" s="14" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
     </row>
     <row r="54">
@@ -1899,7 +1899,7 @@
         </is>
       </c>
       <c r="B54" s="14" t="n">
-        <v>981</v>
+        <v>876</v>
       </c>
       <c r="C54" s="14" t="n">
         <v>2550</v>
@@ -1908,10 +1908,10 @@
         <v>0</v>
       </c>
       <c r="E54" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F54" s="14" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G54" s="14" t="n">
         <v>0</v>
@@ -1924,7 +1924,7 @@
         </is>
       </c>
       <c r="B55" s="14" t="n">
-        <v>983</v>
+        <v>877</v>
       </c>
       <c r="C55" s="14" t="n">
         <v>2550</v>
@@ -1949,7 +1949,7 @@
         </is>
       </c>
       <c r="B56" s="14" t="n">
-        <v>1028.5</v>
+        <v>933.5</v>
       </c>
       <c r="C56" s="14" t="n">
         <v>2550</v>
@@ -1958,10 +1958,10 @@
         <v>0</v>
       </c>
       <c r="E56" s="14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F56" s="14" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G56" s="14" t="n">
         <v>0</v>
@@ -1974,7 +1974,7 @@
         </is>
       </c>
       <c r="B57" s="14" t="n">
-        <v>1037</v>
+        <v>981</v>
       </c>
       <c r="C57" s="14" t="n">
         <v>2550</v>
@@ -1983,10 +1983,10 @@
         <v>0</v>
       </c>
       <c r="E57" s="14" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F57" s="14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G57" s="14" t="n">
         <v>0</v>
@@ -1999,7 +1999,7 @@
         </is>
       </c>
       <c r="B58" s="14" t="n">
-        <v>1078</v>
+        <v>983</v>
       </c>
       <c r="C58" s="14" t="n">
         <v>2550</v>
@@ -2008,7 +2008,7 @@
         <v>0</v>
       </c>
       <c r="E58" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F58" s="14" t="n">
         <v>0</v>
@@ -2024,96 +2024,96 @@
         </is>
       </c>
       <c r="B59" s="14" t="n">
+        <v>1028.5</v>
+      </c>
+      <c r="C59" s="14" t="n">
+        <v>2550</v>
+      </c>
+      <c r="D59" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E59" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F59" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="G59" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="13" t="inlineStr">
+        <is>
+          <t>Plein RDC</t>
+        </is>
+      </c>
+      <c r="B60" s="14" t="n">
+        <v>1037</v>
+      </c>
+      <c r="C60" s="14" t="n">
+        <v>2550</v>
+      </c>
+      <c r="D60" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E60" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="F60" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G60" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="13" t="inlineStr">
+        <is>
+          <t>Plein RDC</t>
+        </is>
+      </c>
+      <c r="B61" s="14" t="n">
+        <v>1078</v>
+      </c>
+      <c r="C61" s="14" t="n">
+        <v>2550</v>
+      </c>
+      <c r="D61" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E61" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F61" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G61" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="13" t="inlineStr">
+        <is>
+          <t>Plein RDC</t>
+        </is>
+      </c>
+      <c r="B62" s="14" t="n">
         <v>1083</v>
       </c>
-      <c r="C59" s="14" t="n">
-        <v>2550</v>
-      </c>
-      <c r="D59" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E59" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="F59" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G59" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="15" t="inlineStr">
-        <is>
-          <t>Dessus fenêtre/porte RDC</t>
-        </is>
-      </c>
-      <c r="B60" s="16" t="n">
-        <v>788</v>
-      </c>
-      <c r="C60" s="16" t="n">
-        <v>749.9</v>
-      </c>
-      <c r="D60" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E60" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F60" s="16" t="n">
-        <v>6</v>
-      </c>
-      <c r="G60" s="16" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="15" t="inlineStr">
-        <is>
-          <t>Dessus fenêtre/porte RDC</t>
-        </is>
-      </c>
-      <c r="B61" s="16" t="n">
-        <v>788</v>
-      </c>
-      <c r="C61" s="16" t="n">
-        <v>750</v>
-      </c>
-      <c r="D61" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E61" s="16" t="n">
-        <v>6</v>
-      </c>
-      <c r="F61" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="G61" s="16" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="15" t="inlineStr">
-        <is>
-          <t>Dessus fenêtre/porte RDC</t>
-        </is>
-      </c>
-      <c r="B62" s="16" t="n">
-        <v>984</v>
-      </c>
-      <c r="C62" s="16" t="n">
-        <v>749.9</v>
-      </c>
-      <c r="D62" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E62" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F62" s="16" t="n">
-        <v>5</v>
-      </c>
-      <c r="G62" s="16" t="n">
+      <c r="C62" s="14" t="n">
+        <v>2550</v>
+      </c>
+      <c r="D62" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E62" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="F62" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G62" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2124,19 +2124,19 @@
         </is>
       </c>
       <c r="B63" s="16" t="n">
-        <v>984</v>
+        <v>788</v>
       </c>
       <c r="C63" s="16" t="n">
-        <v>750</v>
+        <v>749.9</v>
       </c>
       <c r="D63" s="16" t="n">
         <v>0</v>
       </c>
       <c r="E63" s="16" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="F63" s="16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G63" s="16" t="n">
         <v>0</v>
@@ -2149,42 +2149,117 @@
         </is>
       </c>
       <c r="B64" s="16" t="n">
+        <v>788</v>
+      </c>
+      <c r="C64" s="16" t="n">
+        <v>750</v>
+      </c>
+      <c r="D64" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E64" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="F64" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G64" s="16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="15" t="inlineStr">
+        <is>
+          <t>Dessus fenêtre/porte RDC</t>
+        </is>
+      </c>
+      <c r="B65" s="16" t="n">
+        <v>984</v>
+      </c>
+      <c r="C65" s="16" t="n">
+        <v>749.9</v>
+      </c>
+      <c r="D65" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E65" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F65" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="G65" s="16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="15" t="inlineStr">
+        <is>
+          <t>Dessus fenêtre/porte RDC</t>
+        </is>
+      </c>
+      <c r="B66" s="16" t="n">
+        <v>984</v>
+      </c>
+      <c r="C66" s="16" t="n">
+        <v>750</v>
+      </c>
+      <c r="D66" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E66" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="F66" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G66" s="16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="15" t="inlineStr">
+        <is>
+          <t>Dessus fenêtre/porte RDC</t>
+        </is>
+      </c>
+      <c r="B67" s="16" t="n">
         <v>1134</v>
       </c>
-      <c r="C64" s="16" t="n">
+      <c r="C67" s="16" t="n">
         <v>749.9</v>
       </c>
-      <c r="D64" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E64" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F64" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="G64" s="16" t="n">
+      <c r="D67" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E67" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F67" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G67" s="16" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="17" t="inlineStr">
+    <row r="68">
+      <c r="A68" s="17" t="inlineStr">
         <is>
           <t>SURFACE TOTALE (m²)</t>
         </is>
       </c>
-      <c r="B65" s="18" t="n"/>
-      <c r="C65" s="18" t="n"/>
-      <c r="D65" s="19" t="n">
+      <c r="B68" s="18" t="n"/>
+      <c r="C68" s="18" t="n"/>
+      <c r="D68" s="19" t="n">
         <v>88.2641</v>
       </c>
-      <c r="E65" s="19" t="n">
-        <v>149.755</v>
-      </c>
-      <c r="F65" s="19" t="n">
-        <v>157.429</v>
-      </c>
-      <c r="G65" s="19" t="n">
+      <c r="E68" s="19" t="n">
+        <v>172.461</v>
+      </c>
+      <c r="F68" s="19" t="n">
+        <v>183.4954</v>
+      </c>
+      <c r="G68" s="19" t="n">
         <v>83.7351</v>
       </c>
     </row>
@@ -2220,7 +2295,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="18" customHeight="1">
+    <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Catégorie</t>
@@ -2368,7 +2443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2386,7 +2461,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="18" customHeight="1">
+    <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Catégorie</t>
@@ -2441,25 +2516,25 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>Dessus fenêtre N1</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="n">
-        <v>788</v>
-      </c>
-      <c r="C4" s="6" t="n">
-        <v>1008</v>
-      </c>
-      <c r="D4" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="E4" s="25" t="n">
-        <v>0.7943</v>
-      </c>
-      <c r="F4" s="25" t="n">
-        <v>2.3829</v>
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Bandeau Haut</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>4268</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>1064</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E4" s="20" t="n">
+        <v>4.5412</v>
+      </c>
+      <c r="F4" s="20" t="n">
+        <v>22.706</v>
       </c>
     </row>
     <row r="5">
@@ -2469,19 +2544,19 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>984</v>
+        <v>788</v>
       </c>
       <c r="C5" s="6" t="n">
         <v>1008</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E5" s="25" t="n">
-        <v>0.9919</v>
+        <v>0.7943</v>
       </c>
       <c r="F5" s="25" t="n">
-        <v>7.9352</v>
+        <v>2.3829</v>
       </c>
     </row>
     <row r="6">
@@ -2491,41 +2566,41 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>1584</v>
+        <v>984</v>
       </c>
       <c r="C6" s="6" t="n">
         <v>1008</v>
       </c>
       <c r="D6" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="E6" s="25" t="n">
+        <v>0.9919</v>
+      </c>
+      <c r="F6" s="25" t="n">
+        <v>7.9352</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Dessus fenêtre N1</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>1584</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>1008</v>
+      </c>
+      <c r="D7" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E6" s="25" t="n">
+      <c r="E7" s="25" t="n">
         <v>1.5967</v>
       </c>
-      <c r="F6" s="25" t="n">
+      <c r="F7" s="25" t="n">
         <v>4.7901</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>Plein N1</t>
-        </is>
-      </c>
-      <c r="B7" s="8" t="n">
-        <v>445</v>
-      </c>
-      <c r="C7" s="8" t="n">
-        <v>3651.2</v>
-      </c>
-      <c r="D7" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" s="21" t="n">
-        <v>1.6248</v>
-      </c>
-      <c r="F7" s="21" t="n">
-        <v>1.6248</v>
       </c>
     </row>
     <row r="8">
@@ -2535,19 +2610,19 @@
         </is>
       </c>
       <c r="B8" s="8" t="n">
-        <v>491</v>
+        <v>445</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>3650</v>
+        <v>3651.2</v>
       </c>
       <c r="D8" s="8" t="n">
         <v>1</v>
       </c>
       <c r="E8" s="21" t="n">
-        <v>1.7922</v>
+        <v>1.6248</v>
       </c>
       <c r="F8" s="21" t="n">
-        <v>1.7922</v>
+        <v>1.6248</v>
       </c>
     </row>
     <row r="9">
@@ -2557,7 +2632,7 @@
         </is>
       </c>
       <c r="B9" s="8" t="n">
-        <v>620</v>
+        <v>491</v>
       </c>
       <c r="C9" s="8" t="n">
         <v>3650</v>
@@ -2566,10 +2641,10 @@
         <v>1</v>
       </c>
       <c r="E9" s="21" t="n">
-        <v>2.263</v>
+        <v>1.7922</v>
       </c>
       <c r="F9" s="21" t="n">
-        <v>2.263</v>
+        <v>1.7922</v>
       </c>
     </row>
     <row r="10">
@@ -2579,19 +2654,19 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>650.5</v>
+        <v>620</v>
       </c>
       <c r="C10" s="8" t="n">
         <v>3650</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E10" s="21" t="n">
-        <v>2.3743</v>
+        <v>2.263</v>
       </c>
       <c r="F10" s="21" t="n">
-        <v>4.7486</v>
+        <v>2.263</v>
       </c>
     </row>
     <row r="11">
@@ -2601,19 +2676,19 @@
         </is>
       </c>
       <c r="B11" s="8" t="n">
-        <v>778</v>
+        <v>650.5</v>
       </c>
       <c r="C11" s="8" t="n">
         <v>3650</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E11" s="21" t="n">
-        <v>2.8397</v>
+        <v>2.3743</v>
       </c>
       <c r="F11" s="21" t="n">
-        <v>2.8397</v>
+        <v>4.7486</v>
       </c>
     </row>
     <row r="12">
@@ -2623,19 +2698,19 @@
         </is>
       </c>
       <c r="B12" s="8" t="n">
-        <v>821</v>
+        <v>778</v>
       </c>
       <c r="C12" s="8" t="n">
         <v>3650</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E12" s="21" t="n">
-        <v>2.9966</v>
+        <v>2.8397</v>
       </c>
       <c r="F12" s="21" t="n">
-        <v>5.9932</v>
+        <v>2.8397</v>
       </c>
     </row>
     <row r="13">
@@ -2645,19 +2720,19 @@
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>876</v>
+        <v>821</v>
       </c>
       <c r="C13" s="8" t="n">
         <v>3650</v>
       </c>
       <c r="D13" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E13" s="21" t="n">
-        <v>3.1974</v>
+        <v>2.9966</v>
       </c>
       <c r="F13" s="21" t="n">
-        <v>3.1974</v>
+        <v>5.9932</v>
       </c>
     </row>
     <row r="14">
@@ -2667,19 +2742,19 @@
         </is>
       </c>
       <c r="B14" s="8" t="n">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="C14" s="8" t="n">
         <v>3650</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E14" s="21" t="n">
-        <v>3.2011</v>
+        <v>3.1974</v>
       </c>
       <c r="F14" s="21" t="n">
-        <v>6.4022</v>
+        <v>3.1974</v>
       </c>
     </row>
     <row r="15">
@@ -2689,7 +2764,7 @@
         </is>
       </c>
       <c r="B15" s="8" t="n">
-        <v>933.5</v>
+        <v>877</v>
       </c>
       <c r="C15" s="8" t="n">
         <v>3650</v>
@@ -2698,10 +2773,10 @@
         <v>2</v>
       </c>
       <c r="E15" s="21" t="n">
-        <v>3.4073</v>
+        <v>3.2011</v>
       </c>
       <c r="F15" s="21" t="n">
-        <v>6.8146</v>
+        <v>6.4022</v>
       </c>
     </row>
     <row r="16">
@@ -2711,7 +2786,7 @@
         </is>
       </c>
       <c r="B16" s="8" t="n">
-        <v>983</v>
+        <v>933.5</v>
       </c>
       <c r="C16" s="8" t="n">
         <v>3650</v>
@@ -2720,10 +2795,10 @@
         <v>2</v>
       </c>
       <c r="E16" s="21" t="n">
-        <v>3.588</v>
+        <v>3.4073</v>
       </c>
       <c r="F16" s="21" t="n">
-        <v>7.176</v>
+        <v>6.8146</v>
       </c>
     </row>
     <row r="17">
@@ -2733,7 +2808,7 @@
         </is>
       </c>
       <c r="B17" s="8" t="n">
-        <v>1037</v>
+        <v>983</v>
       </c>
       <c r="C17" s="8" t="n">
         <v>3650</v>
@@ -2742,10 +2817,10 @@
         <v>2</v>
       </c>
       <c r="E17" s="21" t="n">
-        <v>3.785</v>
+        <v>3.588</v>
       </c>
       <c r="F17" s="21" t="n">
-        <v>7.57</v>
+        <v>7.176</v>
       </c>
     </row>
     <row r="18">
@@ -2755,19 +2830,19 @@
         </is>
       </c>
       <c r="B18" s="8" t="n">
-        <v>1078</v>
+        <v>1037</v>
       </c>
       <c r="C18" s="8" t="n">
         <v>3650</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E18" s="21" t="n">
-        <v>3.9347</v>
+        <v>3.785</v>
       </c>
       <c r="F18" s="21" t="n">
-        <v>3.9347</v>
+        <v>7.57</v>
       </c>
     </row>
     <row r="19">
@@ -2777,41 +2852,41 @@
         </is>
       </c>
       <c r="B19" s="8" t="n">
+        <v>1078</v>
+      </c>
+      <c r="C19" s="8" t="n">
+        <v>3650</v>
+      </c>
+      <c r="D19" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="21" t="n">
+        <v>3.9347</v>
+      </c>
+      <c r="F19" s="21" t="n">
+        <v>3.9347</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>Plein N1</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="n">
         <v>1083</v>
       </c>
-      <c r="C19" s="8" t="n">
-        <v>3650</v>
-      </c>
-      <c r="D19" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E19" s="21" t="n">
+      <c r="C20" s="8" t="n">
+        <v>3650</v>
+      </c>
+      <c r="D20" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E20" s="21" t="n">
         <v>3.953</v>
       </c>
-      <c r="F19" s="21" t="n">
+      <c r="F20" s="21" t="n">
         <v>7.906</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="9" t="inlineStr">
-        <is>
-          <t>Dessous fenêtre N1</t>
-        </is>
-      </c>
-      <c r="B20" s="10" t="n">
-        <v>788</v>
-      </c>
-      <c r="C20" s="10" t="n">
-        <v>822</v>
-      </c>
-      <c r="D20" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="E20" s="26" t="n">
-        <v>0.6477000000000001</v>
-      </c>
-      <c r="F20" s="26" t="n">
-        <v>3.8862</v>
       </c>
     </row>
     <row r="21">
@@ -2821,41 +2896,41 @@
         </is>
       </c>
       <c r="B21" s="10" t="n">
-        <v>984</v>
+        <v>788</v>
       </c>
       <c r="C21" s="10" t="n">
         <v>822</v>
       </c>
       <c r="D21" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E21" s="26" t="n">
+        <v>0.6477000000000001</v>
+      </c>
+      <c r="F21" s="26" t="n">
+        <v>3.8862</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>Dessous fenêtre N1</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="n">
+        <v>984</v>
+      </c>
+      <c r="C22" s="10" t="n">
+        <v>822</v>
+      </c>
+      <c r="D22" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="E21" s="26" t="n">
+      <c r="E22" s="26" t="n">
         <v>0.8088</v>
       </c>
-      <c r="F21" s="26" t="n">
+      <c r="F22" s="26" t="n">
         <v>6.4704</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="13" t="inlineStr">
-        <is>
-          <t>Plein RDC</t>
-        </is>
-      </c>
-      <c r="B22" s="14" t="n">
-        <v>445</v>
-      </c>
-      <c r="C22" s="14" t="n">
-        <v>2550</v>
-      </c>
-      <c r="D22" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="E22" s="22" t="n">
-        <v>1.1348</v>
-      </c>
-      <c r="F22" s="22" t="n">
-        <v>1.1348</v>
       </c>
     </row>
     <row r="23">
@@ -2865,7 +2940,7 @@
         </is>
       </c>
       <c r="B23" s="14" t="n">
-        <v>491</v>
+        <v>445</v>
       </c>
       <c r="C23" s="14" t="n">
         <v>2550</v>
@@ -2874,10 +2949,10 @@
         <v>1</v>
       </c>
       <c r="E23" s="22" t="n">
-        <v>1.252</v>
+        <v>1.1348</v>
       </c>
       <c r="F23" s="22" t="n">
-        <v>1.252</v>
+        <v>1.1348</v>
       </c>
     </row>
     <row r="24">
@@ -2887,7 +2962,7 @@
         </is>
       </c>
       <c r="B24" s="14" t="n">
-        <v>620</v>
+        <v>491</v>
       </c>
       <c r="C24" s="14" t="n">
         <v>2550</v>
@@ -2896,10 +2971,10 @@
         <v>1</v>
       </c>
       <c r="E24" s="22" t="n">
-        <v>1.581</v>
+        <v>1.252</v>
       </c>
       <c r="F24" s="22" t="n">
-        <v>1.581</v>
+        <v>1.252</v>
       </c>
     </row>
     <row r="25">
@@ -2909,19 +2984,19 @@
         </is>
       </c>
       <c r="B25" s="14" t="n">
-        <v>650.5</v>
+        <v>620</v>
       </c>
       <c r="C25" s="14" t="n">
         <v>2550</v>
       </c>
       <c r="D25" s="14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E25" s="22" t="n">
-        <v>1.6588</v>
+        <v>1.581</v>
       </c>
       <c r="F25" s="22" t="n">
-        <v>3.3176</v>
+        <v>1.581</v>
       </c>
     </row>
     <row r="26">
@@ -2931,19 +3006,19 @@
         </is>
       </c>
       <c r="B26" s="14" t="n">
-        <v>778</v>
+        <v>650.5</v>
       </c>
       <c r="C26" s="14" t="n">
         <v>2550</v>
       </c>
       <c r="D26" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E26" s="22" t="n">
-        <v>1.9839</v>
+        <v>1.6588</v>
       </c>
       <c r="F26" s="22" t="n">
-        <v>1.9839</v>
+        <v>3.3176</v>
       </c>
     </row>
     <row r="27">
@@ -2953,19 +3028,19 @@
         </is>
       </c>
       <c r="B27" s="14" t="n">
-        <v>821</v>
+        <v>778</v>
       </c>
       <c r="C27" s="14" t="n">
         <v>2550</v>
       </c>
       <c r="D27" s="14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E27" s="22" t="n">
-        <v>2.0935</v>
+        <v>1.9839</v>
       </c>
       <c r="F27" s="22" t="n">
-        <v>4.187</v>
+        <v>1.9839</v>
       </c>
     </row>
     <row r="28">
@@ -2975,19 +3050,19 @@
         </is>
       </c>
       <c r="B28" s="14" t="n">
-        <v>876</v>
+        <v>821</v>
       </c>
       <c r="C28" s="14" t="n">
         <v>2550</v>
       </c>
       <c r="D28" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E28" s="22" t="n">
-        <v>2.2338</v>
+        <v>2.0935</v>
       </c>
       <c r="F28" s="22" t="n">
-        <v>2.2338</v>
+        <v>4.187</v>
       </c>
     </row>
     <row r="29">
@@ -2997,19 +3072,19 @@
         </is>
       </c>
       <c r="B29" s="14" t="n">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="C29" s="14" t="n">
         <v>2550</v>
       </c>
       <c r="D29" s="14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E29" s="22" t="n">
-        <v>2.2364</v>
+        <v>2.2338</v>
       </c>
       <c r="F29" s="22" t="n">
-        <v>4.4728</v>
+        <v>2.2338</v>
       </c>
     </row>
     <row r="30">
@@ -3019,7 +3094,7 @@
         </is>
       </c>
       <c r="B30" s="14" t="n">
-        <v>933.5</v>
+        <v>877</v>
       </c>
       <c r="C30" s="14" t="n">
         <v>2550</v>
@@ -3028,10 +3103,10 @@
         <v>2</v>
       </c>
       <c r="E30" s="22" t="n">
-        <v>2.3804</v>
+        <v>2.2364</v>
       </c>
       <c r="F30" s="22" t="n">
-        <v>4.7608</v>
+        <v>4.4728</v>
       </c>
     </row>
     <row r="31">
@@ -3041,7 +3116,7 @@
         </is>
       </c>
       <c r="B31" s="14" t="n">
-        <v>983</v>
+        <v>933.5</v>
       </c>
       <c r="C31" s="14" t="n">
         <v>2550</v>
@@ -3050,10 +3125,10 @@
         <v>2</v>
       </c>
       <c r="E31" s="22" t="n">
-        <v>2.5066</v>
+        <v>2.3804</v>
       </c>
       <c r="F31" s="22" t="n">
-        <v>5.0132</v>
+        <v>4.7608</v>
       </c>
     </row>
     <row r="32">
@@ -3063,7 +3138,7 @@
         </is>
       </c>
       <c r="B32" s="14" t="n">
-        <v>1037</v>
+        <v>983</v>
       </c>
       <c r="C32" s="14" t="n">
         <v>2550</v>
@@ -3072,10 +3147,10 @@
         <v>2</v>
       </c>
       <c r="E32" s="22" t="n">
-        <v>2.6443</v>
+        <v>2.5066</v>
       </c>
       <c r="F32" s="22" t="n">
-        <v>5.2886</v>
+        <v>5.0132</v>
       </c>
     </row>
     <row r="33">
@@ -3085,19 +3160,19 @@
         </is>
       </c>
       <c r="B33" s="14" t="n">
-        <v>1078</v>
+        <v>1037</v>
       </c>
       <c r="C33" s="14" t="n">
         <v>2550</v>
       </c>
       <c r="D33" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E33" s="22" t="n">
-        <v>2.7489</v>
+        <v>2.6443</v>
       </c>
       <c r="F33" s="22" t="n">
-        <v>2.7489</v>
+        <v>5.2886</v>
       </c>
     </row>
     <row r="34">
@@ -3107,41 +3182,41 @@
         </is>
       </c>
       <c r="B34" s="14" t="n">
+        <v>1078</v>
+      </c>
+      <c r="C34" s="14" t="n">
+        <v>2550</v>
+      </c>
+      <c r="D34" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" s="22" t="n">
+        <v>2.7489</v>
+      </c>
+      <c r="F34" s="22" t="n">
+        <v>2.7489</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="13" t="inlineStr">
+        <is>
+          <t>Plein RDC</t>
+        </is>
+      </c>
+      <c r="B35" s="14" t="n">
         <v>1083</v>
       </c>
-      <c r="C34" s="14" t="n">
-        <v>2550</v>
-      </c>
-      <c r="D34" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="E34" s="22" t="n">
+      <c r="C35" s="14" t="n">
+        <v>2550</v>
+      </c>
+      <c r="D35" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="E35" s="22" t="n">
         <v>2.7616</v>
       </c>
-      <c r="F34" s="22" t="n">
+      <c r="F35" s="22" t="n">
         <v>5.5232</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="15" t="inlineStr">
-        <is>
-          <t>Dessus fenêtre/porte RDC</t>
-        </is>
-      </c>
-      <c r="B35" s="16" t="n">
-        <v>788</v>
-      </c>
-      <c r="C35" s="16" t="n">
-        <v>750</v>
-      </c>
-      <c r="D35" s="16" t="n">
-        <v>6</v>
-      </c>
-      <c r="E35" s="27" t="n">
-        <v>0.591</v>
-      </c>
-      <c r="F35" s="27" t="n">
-        <v>3.546</v>
       </c>
     </row>
     <row r="36">
@@ -3151,33 +3226,55 @@
         </is>
       </c>
       <c r="B36" s="16" t="n">
-        <v>984</v>
+        <v>788</v>
       </c>
       <c r="C36" s="16" t="n">
         <v>750</v>
       </c>
       <c r="D36" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="E36" s="27" t="n">
+        <v>0.591</v>
+      </c>
+      <c r="F36" s="27" t="n">
+        <v>3.546</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="15" t="inlineStr">
+        <is>
+          <t>Dessus fenêtre/porte RDC</t>
+        </is>
+      </c>
+      <c r="B37" s="16" t="n">
+        <v>984</v>
+      </c>
+      <c r="C37" s="16" t="n">
+        <v>750</v>
+      </c>
+      <c r="D37" s="16" t="n">
         <v>8</v>
       </c>
-      <c r="E36" s="27" t="n">
+      <c r="E37" s="27" t="n">
         <v>0.738</v>
       </c>
-      <c r="F36" s="27" t="n">
+      <c r="F37" s="27" t="n">
         <v>5.904</v>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="17" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="17" t="inlineStr">
         <is>
           <t>TOTAL FAÇADE</t>
         </is>
       </c>
-      <c r="B37" s="23" t="n"/>
-      <c r="C37" s="23" t="n"/>
-      <c r="D37" s="23" t="n"/>
-      <c r="E37" s="23" t="n"/>
-      <c r="F37" s="24" t="n">
-        <v>149.755</v>
+      <c r="B38" s="23" t="n"/>
+      <c r="C38" s="23" t="n"/>
+      <c r="D38" s="23" t="n"/>
+      <c r="E38" s="23" t="n"/>
+      <c r="F38" s="24" t="n">
+        <v>172.461</v>
       </c>
     </row>
   </sheetData>
@@ -3194,7 +3291,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3212,7 +3309,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="18" customHeight="1">
+    <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Catégorie</t>
@@ -3267,25 +3364,25 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>Dessus fenêtre N1</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="n">
-        <v>788</v>
-      </c>
-      <c r="C4" s="6" t="n">
-        <v>1007.9</v>
-      </c>
-      <c r="D4" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="E4" s="25" t="n">
-        <v>0.7942</v>
-      </c>
-      <c r="F4" s="25" t="n">
-        <v>4.7652</v>
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Bandeau Haut</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>4268</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>1064</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E4" s="20" t="n">
+        <v>4.5412</v>
+      </c>
+      <c r="F4" s="20" t="n">
+        <v>22.706</v>
       </c>
     </row>
     <row r="5">
@@ -3295,41 +3392,41 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>984</v>
+        <v>788</v>
       </c>
       <c r="C5" s="6" t="n">
         <v>1007.9</v>
       </c>
       <c r="D5" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="E5" s="25" t="n">
+        <v>0.7942</v>
+      </c>
+      <c r="F5" s="25" t="n">
+        <v>4.7652</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Dessus fenêtre N1</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>984</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>1007.9</v>
+      </c>
+      <c r="D6" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="E5" s="25" t="n">
+      <c r="E6" s="25" t="n">
         <v>0.9918</v>
       </c>
-      <c r="F5" s="25" t="n">
+      <c r="F6" s="25" t="n">
         <v>4.959</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>Plein N1</t>
-        </is>
-      </c>
-      <c r="B6" s="8" t="n">
-        <v>776</v>
-      </c>
-      <c r="C6" s="8" t="n">
-        <v>3650</v>
-      </c>
-      <c r="D6" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" s="21" t="n">
-        <v>2.8324</v>
-      </c>
-      <c r="F6" s="21" t="n">
-        <v>2.8324</v>
       </c>
     </row>
     <row r="7">
@@ -3339,19 +3436,19 @@
         </is>
       </c>
       <c r="B7" s="8" t="n">
-        <v>777</v>
+        <v>542</v>
       </c>
       <c r="C7" s="8" t="n">
         <v>3650</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E7" s="21" t="n">
-        <v>2.836</v>
+        <v>1.9783</v>
       </c>
       <c r="F7" s="21" t="n">
-        <v>5.672</v>
+        <v>1.9783</v>
       </c>
     </row>
     <row r="8">
@@ -3361,19 +3458,19 @@
         </is>
       </c>
       <c r="B8" s="8" t="n">
-        <v>778</v>
+        <v>776</v>
       </c>
       <c r="C8" s="8" t="n">
         <v>3650</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E8" s="21" t="n">
-        <v>2.8397</v>
+        <v>2.8324</v>
       </c>
       <c r="F8" s="21" t="n">
-        <v>5.6794</v>
+        <v>2.8324</v>
       </c>
     </row>
     <row r="9">
@@ -3383,19 +3480,19 @@
         </is>
       </c>
       <c r="B9" s="8" t="n">
-        <v>822.3</v>
+        <v>777</v>
       </c>
       <c r="C9" s="8" t="n">
         <v>3650</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="E9" s="21" t="n">
-        <v>3.0014</v>
+        <v>2.836</v>
       </c>
       <c r="F9" s="21" t="n">
-        <v>30.014</v>
+        <v>5.672</v>
       </c>
     </row>
     <row r="10">
@@ -3405,19 +3502,19 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>833</v>
+        <v>778</v>
       </c>
       <c r="C10" s="8" t="n">
         <v>3650</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E10" s="21" t="n">
-        <v>3.0404</v>
+        <v>2.8397</v>
       </c>
       <c r="F10" s="21" t="n">
-        <v>12.1616</v>
+        <v>5.6794</v>
       </c>
     </row>
     <row r="11">
@@ -3427,19 +3524,19 @@
         </is>
       </c>
       <c r="B11" s="8" t="n">
-        <v>981</v>
+        <v>822.3</v>
       </c>
       <c r="C11" s="8" t="n">
         <v>3650</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="E11" s="21" t="n">
-        <v>3.5806</v>
+        <v>3.0014</v>
       </c>
       <c r="F11" s="21" t="n">
-        <v>7.1612</v>
+        <v>30.014</v>
       </c>
     </row>
     <row r="12">
@@ -3449,63 +3546,63 @@
         </is>
       </c>
       <c r="B12" s="8" t="n">
+        <v>833</v>
+      </c>
+      <c r="C12" s="8" t="n">
+        <v>3650</v>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="E12" s="21" t="n">
+        <v>3.0404</v>
+      </c>
+      <c r="F12" s="21" t="n">
+        <v>12.1616</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Plein N1</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="n">
+        <v>981</v>
+      </c>
+      <c r="C13" s="8" t="n">
+        <v>3650</v>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E13" s="21" t="n">
+        <v>3.5806</v>
+      </c>
+      <c r="F13" s="21" t="n">
+        <v>7.1612</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Plein N1</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="n">
         <v>1028.5</v>
       </c>
-      <c r="C12" s="8" t="n">
-        <v>3650</v>
-      </c>
-      <c r="D12" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E12" s="21" t="n">
+      <c r="C14" s="8" t="n">
+        <v>3650</v>
+      </c>
+      <c r="D14" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E14" s="21" t="n">
         <v>3.754</v>
       </c>
-      <c r="F12" s="21" t="n">
+      <c r="F14" s="21" t="n">
         <v>7.508</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="9" t="inlineStr">
-        <is>
-          <t>Dessous fenêtre N1</t>
-        </is>
-      </c>
-      <c r="B13" s="10" t="n">
-        <v>788</v>
-      </c>
-      <c r="C13" s="10" t="n">
-        <v>822.1</v>
-      </c>
-      <c r="D13" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="E13" s="26" t="n">
-        <v>0.6478</v>
-      </c>
-      <c r="F13" s="26" t="n">
-        <v>3.8868</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="9" t="inlineStr">
-        <is>
-          <t>Dessous fenêtre N1</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="n">
-        <v>833</v>
-      </c>
-      <c r="C14" s="10" t="n">
-        <v>842.1</v>
-      </c>
-      <c r="D14" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="E14" s="26" t="n">
-        <v>0.7015</v>
-      </c>
-      <c r="F14" s="26" t="n">
-        <v>2.806</v>
       </c>
     </row>
     <row r="15">
@@ -3515,63 +3612,63 @@
         </is>
       </c>
       <c r="B15" s="10" t="n">
-        <v>984</v>
+        <v>788</v>
       </c>
       <c r="C15" s="10" t="n">
         <v>822.1</v>
       </c>
       <c r="D15" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E15" s="26" t="n">
+        <v>0.6478</v>
+      </c>
+      <c r="F15" s="26" t="n">
+        <v>3.8868</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>Dessous fenêtre N1</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="n">
+        <v>833</v>
+      </c>
+      <c r="C16" s="10" t="n">
+        <v>842.1</v>
+      </c>
+      <c r="D16" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E16" s="26" t="n">
+        <v>0.7015</v>
+      </c>
+      <c r="F16" s="26" t="n">
+        <v>2.806</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>Dessous fenêtre N1</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="n">
+        <v>984</v>
+      </c>
+      <c r="C17" s="10" t="n">
+        <v>822.1</v>
+      </c>
+      <c r="D17" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="E15" s="26" t="n">
+      <c r="E17" s="26" t="n">
         <v>0.8089</v>
       </c>
-      <c r="F15" s="26" t="n">
+      <c r="F17" s="26" t="n">
         <v>4.0445</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="13" t="inlineStr">
-        <is>
-          <t>Plein RDC</t>
-        </is>
-      </c>
-      <c r="B16" s="14" t="n">
-        <v>776</v>
-      </c>
-      <c r="C16" s="14" t="n">
-        <v>2550</v>
-      </c>
-      <c r="D16" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="E16" s="22" t="n">
-        <v>1.9788</v>
-      </c>
-      <c r="F16" s="22" t="n">
-        <v>1.9788</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="13" t="inlineStr">
-        <is>
-          <t>Plein RDC</t>
-        </is>
-      </c>
-      <c r="B17" s="14" t="n">
-        <v>777</v>
-      </c>
-      <c r="C17" s="14" t="n">
-        <v>2550</v>
-      </c>
-      <c r="D17" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="E17" s="22" t="n">
-        <v>1.9814</v>
-      </c>
-      <c r="F17" s="22" t="n">
-        <v>3.9628</v>
       </c>
     </row>
     <row r="18">
@@ -3581,19 +3678,19 @@
         </is>
       </c>
       <c r="B18" s="14" t="n">
-        <v>778</v>
+        <v>542</v>
       </c>
       <c r="C18" s="14" t="n">
         <v>2550</v>
       </c>
       <c r="D18" s="14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E18" s="22" t="n">
-        <v>1.9839</v>
+        <v>1.3821</v>
       </c>
       <c r="F18" s="22" t="n">
-        <v>3.9678</v>
+        <v>1.3821</v>
       </c>
     </row>
     <row r="19">
@@ -3603,19 +3700,19 @@
         </is>
       </c>
       <c r="B19" s="14" t="n">
-        <v>822.3</v>
+        <v>776</v>
       </c>
       <c r="C19" s="14" t="n">
         <v>2550</v>
       </c>
       <c r="D19" s="14" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E19" s="22" t="n">
-        <v>2.0969</v>
+        <v>1.9788</v>
       </c>
       <c r="F19" s="22" t="n">
-        <v>20.969</v>
+        <v>1.9788</v>
       </c>
     </row>
     <row r="20">
@@ -3625,19 +3722,19 @@
         </is>
       </c>
       <c r="B20" s="14" t="n">
-        <v>833</v>
+        <v>777</v>
       </c>
       <c r="C20" s="14" t="n">
         <v>2550</v>
       </c>
       <c r="D20" s="14" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E20" s="22" t="n">
-        <v>2.1242</v>
+        <v>1.9814</v>
       </c>
       <c r="F20" s="22" t="n">
-        <v>8.4968</v>
+        <v>3.9628</v>
       </c>
     </row>
     <row r="21">
@@ -3647,7 +3744,7 @@
         </is>
       </c>
       <c r="B21" s="14" t="n">
-        <v>981</v>
+        <v>778</v>
       </c>
       <c r="C21" s="14" t="n">
         <v>2550</v>
@@ -3656,10 +3753,10 @@
         <v>2</v>
       </c>
       <c r="E21" s="22" t="n">
-        <v>2.5016</v>
+        <v>1.9839</v>
       </c>
       <c r="F21" s="22" t="n">
-        <v>5.0032</v>
+        <v>3.9678</v>
       </c>
     </row>
     <row r="22">
@@ -3669,77 +3766,143 @@
         </is>
       </c>
       <c r="B22" s="14" t="n">
+        <v>822.3</v>
+      </c>
+      <c r="C22" s="14" t="n">
+        <v>2550</v>
+      </c>
+      <c r="D22" s="14" t="n">
+        <v>10</v>
+      </c>
+      <c r="E22" s="22" t="n">
+        <v>2.0969</v>
+      </c>
+      <c r="F22" s="22" t="n">
+        <v>20.969</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>Plein RDC</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="n">
+        <v>833</v>
+      </c>
+      <c r="C23" s="14" t="n">
+        <v>2550</v>
+      </c>
+      <c r="D23" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="E23" s="22" t="n">
+        <v>2.1242</v>
+      </c>
+      <c r="F23" s="22" t="n">
+        <v>8.4968</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="13" t="inlineStr">
+        <is>
+          <t>Plein RDC</t>
+        </is>
+      </c>
+      <c r="B24" s="14" t="n">
+        <v>981</v>
+      </c>
+      <c r="C24" s="14" t="n">
+        <v>2550</v>
+      </c>
+      <c r="D24" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="E24" s="22" t="n">
+        <v>2.5016</v>
+      </c>
+      <c r="F24" s="22" t="n">
+        <v>5.0032</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>Plein RDC</t>
+        </is>
+      </c>
+      <c r="B25" s="14" t="n">
         <v>1028.5</v>
       </c>
-      <c r="C22" s="14" t="n">
-        <v>2550</v>
-      </c>
-      <c r="D22" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="E22" s="22" t="n">
+      <c r="C25" s="14" t="n">
+        <v>2550</v>
+      </c>
+      <c r="D25" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="E25" s="22" t="n">
         <v>2.6227</v>
       </c>
-      <c r="F22" s="22" t="n">
+      <c r="F25" s="22" t="n">
         <v>5.2454</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="15" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="15" t="inlineStr">
         <is>
           <t>Dessus fenêtre/porte RDC</t>
         </is>
       </c>
-      <c r="B23" s="16" t="n">
+      <c r="B26" s="16" t="n">
         <v>788</v>
       </c>
-      <c r="C23" s="16" t="n">
+      <c r="C26" s="16" t="n">
         <v>749.9</v>
       </c>
-      <c r="D23" s="16" t="n">
+      <c r="D26" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="E23" s="27" t="n">
+      <c r="E26" s="27" t="n">
         <v>0.5909</v>
       </c>
-      <c r="F23" s="27" t="n">
+      <c r="F26" s="27" t="n">
         <v>3.5454</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="15" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="15" t="inlineStr">
         <is>
           <t>Dessus fenêtre/porte RDC</t>
         </is>
       </c>
-      <c r="B24" s="16" t="n">
+      <c r="B27" s="16" t="n">
         <v>984</v>
       </c>
-      <c r="C24" s="16" t="n">
+      <c r="C27" s="16" t="n">
         <v>749.9</v>
       </c>
-      <c r="D24" s="16" t="n">
+      <c r="D27" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="E24" s="27" t="n">
+      <c r="E27" s="27" t="n">
         <v>0.7379</v>
       </c>
-      <c r="F24" s="27" t="n">
+      <c r="F27" s="27" t="n">
         <v>3.6895</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="17" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="17" t="inlineStr">
         <is>
           <t>TOTAL FAÇADE</t>
         </is>
       </c>
-      <c r="B25" s="23" t="n"/>
-      <c r="C25" s="23" t="n"/>
-      <c r="D25" s="23" t="n"/>
-      <c r="E25" s="23" t="n"/>
-      <c r="F25" s="24" t="n">
-        <v>157.429</v>
+      <c r="B28" s="23" t="n"/>
+      <c r="C28" s="23" t="n"/>
+      <c r="D28" s="23" t="n"/>
+      <c r="E28" s="23" t="n"/>
+      <c r="F28" s="24" t="n">
+        <v>183.4954</v>
       </c>
     </row>
   </sheetData>
@@ -3774,7 +3937,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="18" customHeight="1">
+    <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Catégorie</t>

</xml_diff>